<commit_message>
transport-mode: fix candidate release 2.0.0
</commit_message>
<xml_diff>
--- a/transport-mode/transport-mode.xlsx
+++ b/transport-mode/transport-mode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scrocca\Desktop\cefriel-github\controlled-vocabularies\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5926D73A-9D3B-4B26-A78E-54F80287A89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3B11E8-9877-4033-A576-1A0FFA05F08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="393">
   <si>
     <t>ConceptScheme URI</t>
   </si>
@@ -1371,6 +1371,9 @@
   </si>
   <si>
     <t>Draft Controlled Vocabulary</t>
+  </si>
+  <si>
+    <t>skos:narrower</t>
   </si>
 </sst>
 </file>
@@ -1536,7 +1539,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1588,9 +1591,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1599,9 +1599,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1613,6 +1610,27 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1933,16 +1951,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="60.28515625" customWidth="1"/>
     <col min="3" max="3" width="85.28515625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="71.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="35.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="30.42578125" customWidth="1"/>
-    <col min="7" max="7" width="55.28515625" customWidth="1"/>
+    <col min="4" max="5" width="71.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="35.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" customWidth="1"/>
+    <col min="8" max="8" width="55.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2088,324 +2106,352 @@
         <v>391</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="38" t="s">
         <v>26</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" s="14" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="str">
         <f t="shared" ref="A20:A58" si="0">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B20)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/road-transport</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D20" s="37" t="str">
+        <f>_xlfn.TEXTJOIN(",",,A21:A25)</f>
+        <v>https://w3id.org/mobilitydcat-ap/transport-mode/car,https://w3id.org/mobilitydcat-ap/transport-mode/motorcycle,https://w3id.org/mobilitydcat-ap/transport-mode/bus,https://w3id.org/mobilitydcat-ap/transport-mode/coach,https://w3id.org/mobilitydcat-ap/transport-mode/truck</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f t="shared" ref="A21:A28" si="1">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B21)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="37" t="s">
+      <c r="C21" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D21"/>
+      <c r="E21" t="str">
         <f>A20</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/road-transport</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/motorcycle</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D22"/>
+      <c r="E22" t="str">
         <f>A20</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/road-transport</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/bus</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="C23" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="D23" t="str">
+      <c r="D23"/>
+      <c r="E23" t="str">
         <f>A20</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/road-transport</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/coach</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="34" t="s">
         <v>42</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="14" t="str">
+      <c r="E24" s="14" t="str">
         <f>A20</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/road-transport</v>
       </c>
-      <c r="E24" s="15"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F24" s="15"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/truck</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="37" t="s">
+      <c r="C25" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="D25" t="str">
+      <c r="D25"/>
+      <c r="E25" t="str">
         <f>A20</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/road-transport</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" s="14" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="28" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/rail-transport</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="39" t="s">
         <v>47</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="15"/>
+      <c r="D26" s="15" t="str">
+        <f>_xlfn.TEXTJOIN(",",,A27:A29,A31)</f>
+        <v>https://w3id.org/mobilitydcat-ap/transport-mode/long-distance-rail,https://w3id.org/mobilitydcat-ap/transport-mode/regional-and-local-rail,https://w3id.org/mobilitydcat-ap/transport-mode/tram-light-rail,https://w3id.org/mobilitydcat-ap/transport-mode/metro</v>
+      </c>
       <c r="E26" s="15"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F26" s="15"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/long-distance-rail</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="37" t="s">
+      <c r="C27" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="D27" s="1" t="str">
+      <c r="E27" s="1" t="str">
         <f>A26</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/rail-transport</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="33" t="str">
+    <row r="28" spans="1:8" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="32" t="str">
         <f t="shared" si="1"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/regional-and-local-rail</v>
       </c>
-      <c r="B28" s="34" t="s">
+      <c r="B28" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="37" t="s">
+      <c r="C28" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="1" t="str">
+      <c r="D28" s="1"/>
+      <c r="E28" s="1" t="str">
         <f>A26</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/rail-transport</v>
       </c>
-      <c r="E28" s="32"/>
-    </row>
-    <row r="29" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F28" s="31"/>
+    </row>
+    <row r="29" spans="1:8" s="32" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="37" t="s">
+      <c r="B29" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="37" t="s">
+      <c r="C29" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="32" t="str">
+      <c r="D29" s="31"/>
+      <c r="E29" s="31" t="str">
         <f>A26</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/rail-transport</v>
       </c>
-      <c r="E29" s="32"/>
-    </row>
-    <row r="30" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="31"/>
+    </row>
+    <row r="30" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="str">
         <f t="shared" ref="A30:A36" si="2">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B30)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/metro-subway-train</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="43" t="s">
         <v>61</v>
       </c>
       <c r="C30" s="10"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
-      <c r="F30" s="9" t="b">
+      <c r="F30" s="16"/>
+      <c r="G30" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G30" s="9" t="str">
+      <c r="H30" s="9" t="str">
         <f>A31</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/metro</v>
       </c>
     </row>
-    <row r="31" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="str">
         <f t="shared" si="2"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/metro</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="34" t="s">
         <v>62</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="D31" s="15" t="str">
+      <c r="D31" s="15"/>
+      <c r="E31" s="15" t="str">
         <f>A26</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/rail-transport</v>
       </c>
-      <c r="E31" s="15"/>
-    </row>
-    <row r="32" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F31" s="15"/>
+    </row>
+    <row r="32" spans="1:8" s="14" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="str">
         <f t="shared" si="2"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/water-transport</v>
       </c>
-      <c r="B32" s="29" t="s">
+      <c r="B32" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="15"/>
+      <c r="D32" s="15" t="str">
+        <f>_xlfn.TEXTJOIN(",",,A33:A36)</f>
+        <v>https://w3id.org/mobilitydcat-ap/transport-mode/maritime,https://w3id.org/mobilitydcat-ap/transport-mode/inland-waterways,https://w3id.org/mobilitydcat-ap/transport-mode/shuttle-ferry,https://w3id.org/mobilitydcat-ap/transport-mode/water-taxi</v>
+      </c>
       <c r="E32" s="15"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F32" s="15"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f t="shared" si="2"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/maritime</v>
       </c>
-      <c r="B33" s="34" t="s">
+      <c r="B33" s="41" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="37" t="s">
+      <c r="C33" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="1" t="str">
+      <c r="E33" s="1" t="str">
         <f>A32</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/water-transport</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="str">
         <f t="shared" si="2"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/inland-waterways</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="34" t="s">
         <v>68</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="D34" s="1" t="str">
+      <c r="E34" s="1" t="str">
         <f>A32</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/water-transport</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f t="shared" si="2"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/shuttle-ferry</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="C35" s="37" t="s">
+      <c r="C35" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="D35" s="1" t="str">
+      <c r="E35" s="1" t="str">
         <f>A32</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/water-transport</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="str">
         <f t="shared" si="2"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/water-taxi</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="35" t="s">
+      <c r="C36" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="D36" s="15" t="str">
+      <c r="D36" s="15"/>
+      <c r="E36" s="15" t="str">
         <f>A32</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/water-transport</v>
       </c>
-      <c r="E36" s="15"/>
-    </row>
-    <row r="37" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F36" s="15"/>
+    </row>
+    <row r="37" spans="1:8" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="28" t="str">
         <f t="shared" ref="A37" si="3">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B37)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/air-transport</v>
       </c>
-      <c r="B37" s="29" t="s">
+      <c r="B37" s="39" t="s">
         <v>75</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="15"/>
+      <c r="D37" s="15" t="str">
+        <f>_xlfn.TEXTJOIN(",",,A39:A40)</f>
+        <v>https://w3id.org/mobilitydcat-ap/transport-mode/aeroplane,https://w3id.org/mobilitydcat-ap/transport-mode/air-taxi</v>
+      </c>
       <c r="E37" s="15"/>
-    </row>
-    <row r="38" spans="1:7" s="9" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F37" s="15"/>
+    </row>
+    <row r="38" spans="1:8" s="9" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/air</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="43" t="s">
         <v>77</v>
       </c>
       <c r="C38" s="10" t="s">
@@ -2413,337 +2459,358 @@
       </c>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
-      <c r="F38" s="9" t="b">
+      <c r="F38" s="16"/>
+      <c r="G38" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G38" s="9" t="str">
+      <c r="H38" s="9" t="str">
         <f>A37</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/air-transport</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B39)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/aeroplane</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="34" t="s">
         <v>78</v>
       </c>
       <c r="C39" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="1" t="str">
+      <c r="E39" s="1" t="str">
         <f>A37</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/air-transport</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="str">
         <f t="shared" ref="A40" si="4">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B40)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/air-taxi</v>
       </c>
-      <c r="B40" s="36" t="s">
+      <c r="B40" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="C40" s="35" t="s">
+      <c r="C40" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="D40" s="1" t="str">
+      <c r="E40" s="1" t="str">
         <f>A37</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/air-transport</v>
       </c>
     </row>
-    <row r="41" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
+    <row r="41" spans="1:8" s="14" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A41" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="39" t="s">
         <v>89</v>
       </c>
       <c r="C41" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="D41" s="15"/>
+      <c r="D41" s="15" t="str">
+        <f>_xlfn.TEXTJOIN(",",,A42:A45)</f>
+        <v>https://w3id.org/mobilitydcat-ap/transport-mode/cableways,https://w3id.org/mobilitydcat-ap/transport-mode/elevator,https://w3id.org/mobilitydcat-ap/transport-mode/escalator,https://w3id.org/mobilitydcat-ap/transport-mode/seasonal-transport</v>
+      </c>
       <c r="E41" s="15"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F41" s="15"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B42)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/cableways</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="34" t="s">
         <v>91</v>
       </c>
       <c r="C42" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="D42" t="str">
+      <c r="D42"/>
+      <c r="E42" t="str">
         <f>A41</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/special-transport</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B43" s="13" t="s">
+      <c r="B43" s="34" t="s">
         <v>94</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="D43" s="1" t="str">
+      <c r="E43" s="1" t="str">
         <f>A41</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/special-transport</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="34" t="s">
         <v>97</v>
       </c>
       <c r="C44" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="D44" s="1" t="str">
+      <c r="E44" s="1" t="str">
         <f>A41</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/special-transport</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B45)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/seasonal-transport</v>
       </c>
-      <c r="B45" s="13" t="s">
+      <c r="B45" s="34" t="s">
         <v>99</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="D45" s="15" t="str">
+      <c r="D45" s="15"/>
+      <c r="E45" s="15" t="str">
         <f>A41</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/special-transport</v>
       </c>
-      <c r="E45" s="15"/>
-    </row>
-    <row r="46" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F45" s="15"/>
+    </row>
+    <row r="46" spans="1:8" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A46" s="28" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B46)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/micromobility</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B46" s="39" t="s">
         <v>101</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="D46" s="15"/>
+      <c r="D46" s="15" t="str">
+        <f>_xlfn.TEXTJOIN(",",,A47:A49)</f>
+        <v>https://w3id.org/mobilitydcat-ap/transport-mode/bicycle,https://w3id.org/mobilitydcat-ap/transport-mode/e-scooter,https://w3id.org/mobilitydcat-ap/transport-mode/moped</v>
+      </c>
       <c r="E46" s="15"/>
-    </row>
-    <row r="47" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F46" s="15"/>
+    </row>
+    <row r="47" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>103</v>
       </c>
-      <c r="B47" s="37" t="s">
+      <c r="B47" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="C47" s="37" t="s">
+      <c r="C47" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="D47" s="1" t="str">
+      <c r="E47" s="1" t="str">
         <f>A46</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/micromobility</v>
       </c>
     </row>
-    <row r="48" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B48)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/e-scooter</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="34" t="s">
         <v>106</v>
       </c>
       <c r="C48" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="15" t="str">
+      <c r="D48" s="15"/>
+      <c r="E48" s="15" t="str">
         <f>A46</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/micromobility</v>
       </c>
-      <c r="E48" s="15"/>
-    </row>
-    <row r="49" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F48" s="15"/>
+    </row>
+    <row r="49" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B49)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/moped</v>
       </c>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="34" t="s">
         <v>108</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="D49" s="15" t="str">
+      <c r="D49" s="15"/>
+      <c r="E49" s="15" t="str">
         <f>A46</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/micromobility</v>
       </c>
-      <c r="E49" s="15"/>
-    </row>
-    <row r="50" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="31" t="str">
+      <c r="F49" s="15"/>
+    </row>
+    <row r="50" spans="1:8" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="30" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B50)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/pedestrian</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="39" t="s">
         <v>110</v>
       </c>
       <c r="C50" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="D50" s="32"/>
-      <c r="E50" s="32"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D50" s="31"/>
+      <c r="E50" s="31"/>
+      <c r="F50" s="31"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B51)," ","-"),",",""))</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/other</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="39" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="52" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/bike-hire</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B52" s="43" t="s">
         <v>113</v>
       </c>
       <c r="C52" s="10"/>
       <c r="D52" s="16"/>
       <c r="E52" s="16"/>
-      <c r="F52" s="9" t="b">
+      <c r="F52" s="16"/>
+      <c r="G52" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G52" s="9" t="str">
+      <c r="H52" s="9" t="str">
         <f>A47</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/bicycle</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/bike-sharing</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="43" t="s">
         <v>114</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="16"/>
       <c r="E53" s="16"/>
-      <c r="F53" s="9" t="b">
+      <c r="F53" s="16"/>
+      <c r="G53" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G53" s="9" t="str">
+      <c r="H53" s="9" t="str">
         <f>A47</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/bicycle</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car-hire</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="B54" s="43" t="s">
         <v>115</v>
       </c>
       <c r="C54" s="10"/>
       <c r="D54" s="16"/>
       <c r="E54" s="16"/>
-      <c r="F54" s="9" t="b">
+      <c r="F54" s="16"/>
+      <c r="G54" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G54" s="9" t="str">
+      <c r="H54" s="9" t="str">
         <f>A21</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car-pooling</v>
       </c>
-      <c r="B55" s="10" t="s">
+      <c r="B55" s="43" t="s">
         <v>116</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="16"/>
       <c r="E55" s="16"/>
-      <c r="F55" s="9" t="b">
+      <c r="F55" s="16"/>
+      <c r="G55" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G55" s="9" t="str">
+      <c r="H55" s="9" t="str">
         <f>A21</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car-sharing</v>
       </c>
-      <c r="B56" s="10" t="s">
+      <c r="B56" s="43" t="s">
         <v>117</v>
       </c>
       <c r="C56" s="10"/>
       <c r="D56" s="16"/>
       <c r="E56" s="16"/>
-      <c r="F56" s="9" t="b">
+      <c r="F56" s="16"/>
+      <c r="G56" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G56" s="9" t="str">
+      <c r="H56" s="9" t="str">
         <f>A21</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/ride-pooling</v>
       </c>
-      <c r="B57" s="10" t="s">
+      <c r="B57" s="43" t="s">
         <v>118</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="16"/>
       <c r="E57" s="16"/>
-      <c r="F57" s="9" t="b">
+      <c r="F57" s="16"/>
+      <c r="G57" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G57" s="9" t="str">
+      <c r="H57" s="9" t="str">
         <f>A21</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/taxi</v>
       </c>
-      <c r="B58" s="10" t="s">
+      <c r="B58" s="43" t="s">
         <v>119</v>
       </c>
       <c r="C58" s="10"/>
       <c r="D58" s="16"/>
       <c r="E58" s="16"/>
-      <c r="F58" s="9" t="b">
+      <c r="F58" s="16"/>
+      <c r="G58" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G58" s="9" t="str">
+      <c r="H58" s="9" t="str">
         <f>A21</f>
         <v>https://w3id.org/mobilitydcat-ap/transport-mode/car</v>
       </c>
@@ -4479,14 +4546,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4691,21 +4756,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00E07F1C-30C1-44FD-9041-9A393B69CD1A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E852E-38F4-443F-ABCC-E4BE2043727A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
-    <ds:schemaRef ds:uri="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4730,9 +4794,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E852E-38F4-443F-ABCC-E4BE2043727A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00E07F1C-30C1-44FD-9041-9A393B69CD1A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
+    <ds:schemaRef ds:uri="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>